<commit_message>
Add Mil Med sleep quality publication and drop ahead-of-print labels
Added Hoch JM et al. (2026) "The Relationship Between Sleep Quality,
Pain, and Health-Related Quality of Life in Entry-Level Marines" to
published articles. Removed the "ahead of print" label from the Porter
et al. (2025) Mil Med entry so epub entries carry only the DOI.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/cv.xlsx
+++ b/data/cv.xlsx
@@ -365,7 +365,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:H24"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="20.7109375" style="2" customWidth="1"/>
@@ -1087,11 +1087,6 @@
           <t>Military Medicine</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>ahead of print</t>
-        </is>
-      </c>
       <c r="H21" t="inlineStr">
         <is>
           <t>10.1093/milmed/usaf493</t>
@@ -1166,6 +1161,39 @@
       <c r="H23" t="inlineStr">
         <is>
           <t>10.1080/1091367X.2026.2692042</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>peer_rev_pub_article</t>
+        </is>
+      </c>
+      <c r="B24" s="2">
+        <v>46224</v>
+      </c>
+      <c r="C24">
+        <v>2026</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Hoch JM, Dlugonski D, Cramer RJ, **Bergin RT**, Torp DM, Heimark McCloughan N, Green B, Sessoms PH, Fraser JJ, Hoch MC</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>The Relationship Between Sleep Quality, Pain, and Health-Related Quality of Life in Entry-Level Marines</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Military Medicine</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>10.1093/milmed/usag318</t>
         </is>
       </c>
     </row>

</xml_diff>